<commit_message>
added results to the data points
</commit_message>
<xml_diff>
--- a/map_data.xlsx
+++ b/map_data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
   <si>
     <t xml:space="preserve">Sample</t>
   </si>
@@ -43,7 +43,7 @@
     <t xml:space="preserve">18.393109</t>
   </si>
   <si>
-    <t xml:space="preserve">okänd</t>
+    <t xml:space="preserve">negativ</t>
   </si>
   <si>
     <t xml:space="preserve">Skullersta</t>
@@ -71,6 +71,9 @@
   </si>
   <si>
     <t xml:space="preserve">17.688138</t>
+  </si>
+  <si>
+    <t xml:space="preserve">positiv</t>
   </si>
   <si>
     <t xml:space="preserve">Nora</t>
@@ -208,13 +211,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -427,142 +434,142 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="0" t="s">
-        <v>7</v>
+      <c r="D5" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="0" t="s">
+      <c r="A11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="B11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="C11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added details about replicates to data points
</commit_message>
<xml_diff>
--- a/map_data.xlsx
+++ b/map_data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
   <si>
     <t xml:space="preserve">Sample</t>
   </si>
@@ -34,6 +34,9 @@
     <t xml:space="preserve">Result</t>
   </si>
   <si>
+    <t xml:space="preserve">Details</t>
+  </si>
+  <si>
     <t xml:space="preserve">Näs</t>
   </si>
   <si>
@@ -46,6 +49,9 @@
     <t xml:space="preserve">negativ</t>
   </si>
   <si>
+    <t xml:space="preserve">(0/3)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Skullersta</t>
   </si>
   <si>
@@ -76,6 +82,9 @@
     <t xml:space="preserve">positiv</t>
   </si>
   <si>
+    <t xml:space="preserve">(2/3)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nora</t>
   </si>
   <si>
@@ -119,6 +128,9 @@
   </si>
   <si>
     <t xml:space="preserve">17.902287</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1/3)</t>
   </si>
   <si>
     <t xml:space="preserve">Häggvik</t>
@@ -416,7 +428,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -432,145 +444,178 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added a clickable interactive table on the left hand side
</commit_message>
<xml_diff>
--- a/map_data.xlsx
+++ b/map_data.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
   <si>
-    <t xml:space="preserve">Sample</t>
+    <t xml:space="preserve">Prov</t>
   </si>
   <si>
     <t xml:space="preserve">Latitude</t>
@@ -31,10 +31,10 @@
     <t xml:space="preserve">Longitude</t>
   </si>
   <si>
-    <t xml:space="preserve">Result</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Details</t>
+    <t xml:space="preserve">Resultat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replikat</t>
   </si>
   <si>
     <t xml:space="preserve">Näs</t>
@@ -461,7 +461,7 @@
       <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -478,7 +478,7 @@
       <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -495,7 +495,7 @@
       <c r="D4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -512,7 +512,7 @@
       <c r="D5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -529,7 +529,7 @@
       <c r="D6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -546,7 +546,7 @@
       <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -563,7 +563,7 @@
       <c r="D8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -580,7 +580,7 @@
       <c r="D9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -597,7 +597,7 @@
       <c r="D10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" s="2" t="s">
         <v>36</v>
       </c>
     </row>
@@ -614,7 +614,7 @@
       <c r="D11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" s="2" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added filtering parameters to the map
</commit_message>
<xml_diff>
--- a/map_data.xlsx
+++ b/map_data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="43">
   <si>
     <t xml:space="preserve">Prov</t>
   </si>
@@ -37,6 +37,12 @@
     <t xml:space="preserve">Replikat</t>
   </si>
   <si>
+    <t xml:space="preserve">Datum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provomgång</t>
+  </si>
+  <si>
     <t xml:space="preserve">Näs</t>
   </si>
   <si>
@@ -50,6 +56,9 @@
   </si>
   <si>
     <t xml:space="preserve">(0/3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">244-2026</t>
   </si>
   <si>
     <t xml:space="preserve">Skullersta</t>
@@ -428,7 +437,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -447,175 +456,211 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>36</v>
+        <v>39</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>